<commit_message>
Update CW data 2026-08-31
</commit_message>
<xml_diff>
--- a/docs/downloads/KetQuaGiaoDich_latest.xlsx
+++ b/docs/downloads/KetQuaGiaoDich_latest.xlsx
@@ -573,7 +573,7 @@
         <v>8.06</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
     </row>
@@ -609,7 +609,7 @@
         <v>328.36</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
     </row>
@@ -645,7 +645,7 @@
         <v>18.76</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
     </row>
@@ -677,7 +677,7 @@
         <v>38.63</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
     </row>
@@ -713,7 +713,7 @@
         <v>16.84</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
     </row>
@@ -749,7 +749,7 @@
         <v>29.19</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
     </row>
@@ -785,7 +785,7 @@
         <v>11.32</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
     </row>
@@ -821,7 +821,7 @@
         <v>12.51</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
     </row>
@@ -857,7 +857,7 @@
         <v>7.91</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
     </row>
@@ -893,7 +893,7 @@
         <v>8.01</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
     </row>
@@ -929,7 +929,7 @@
         <v>10.18</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
     </row>
@@ -961,7 +961,7 @@
         <v>21.02</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
     </row>
@@ -993,7 +993,7 @@
         <v>20.21</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
     </row>
@@ -1025,7 +1025,7 @@
         <v>13.83</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
     </row>
@@ -1061,7 +1061,7 @@
         <v>27.37</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         <v>437.98</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
     </row>
@@ -1129,7 +1129,7 @@
         <v>12.65</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
     </row>
@@ -1161,7 +1161,7 @@
         <v>6.15</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
     </row>
@@ -1197,7 +1197,7 @@
         <v>11.8</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
     </row>
@@ -1233,7 +1233,7 @@
         <v>12.72</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
     </row>
@@ -1269,7 +1269,7 @@
         <v>10.89</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
     </row>
@@ -1301,7 +1301,7 @@
         <v>850.29</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
     </row>
@@ -1337,7 +1337,7 @@
         <v>462.26</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
     </row>
@@ -1373,7 +1373,7 @@
         <v>23.71</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
     </row>
@@ -1409,7 +1409,7 @@
         <v>205.45</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
     </row>
@@ -1445,7 +1445,7 @@
         <v>30.82</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
     </row>
@@ -1481,7 +1481,7 @@
         <v>371.04</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
     </row>
@@ -1513,7 +1513,7 @@
         <v>37.1</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
     </row>
@@ -1549,7 +1549,7 @@
         <v>29.68</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
     </row>
@@ -1581,7 +1581,7 @@
         <v>371.04</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
     </row>
@@ -1613,7 +1613,7 @@
         <v>742.08</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
     </row>
@@ -1645,7 +1645,7 @@
         <v>23.19</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
     </row>
@@ -1681,7 +1681,7 @@
         <v>16.27</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         <v>5.9</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
     </row>
@@ -1753,7 +1753,7 @@
         <v>6.12</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
     </row>
@@ -1789,7 +1789,7 @@
         <v>19.26</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
     </row>
@@ -1825,7 +1825,7 @@
         <v>11.26</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
     </row>
@@ -1861,7 +1861,7 @@
         <v>7.21</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
     </row>
@@ -1897,7 +1897,7 @@
         <v>12.04</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
     </row>
@@ -1933,7 +1933,7 @@
         <v>10.64</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
     </row>
@@ -1969,7 +1969,7 @@
         <v>25.79</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
     </row>
@@ -2005,7 +2005,7 @@
         <v>75.20999999999999</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
     </row>
@@ -2037,7 +2037,7 @@
         <v>902.5</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
     </row>
@@ -2073,7 +2073,7 @@
         <v>7.97</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
     </row>
@@ -2109,7 +2109,7 @@
         <v>6.78</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
     </row>
@@ -2145,7 +2145,7 @@
         <v>6.78</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
     </row>
@@ -2181,7 +2181,7 @@
         <v>5.4</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
     </row>
@@ -2217,7 +2217,7 @@
         <v>9.890000000000001</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
     </row>
@@ -2253,7 +2253,7 @@
         <v>7.47</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
     </row>
@@ -2289,7 +2289,7 @@
         <v>4.09</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
     </row>
@@ -2325,7 +2325,7 @@
         <v>4.52</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
     </row>
@@ -2361,7 +2361,7 @@
         <v>30.05</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
     </row>
@@ -2397,7 +2397,7 @@
         <v>6.43</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
     </row>
@@ -2433,7 +2433,7 @@
         <v>29.89</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
     </row>
@@ -2469,7 +2469,7 @@
         <v>5.19</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
     </row>
@@ -2505,7 +2505,7 @@
         <v>12.69</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
     </row>
@@ -2541,7 +2541,7 @@
         <v>9</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
     </row>
@@ -2577,7 +2577,7 @@
         <v>18.53</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
     </row>
@@ -2613,7 +2613,7 @@
         <v>10.22</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
     </row>
@@ -2649,7 +2649,7 @@
         <v>4.79</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
     </row>
@@ -2685,7 +2685,7 @@
         <v>3.34</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
     </row>
@@ -2717,7 +2717,7 @@
         <v>10.18</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
     </row>
@@ -2753,7 +2753,7 @@
         <v>8.42</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
     </row>
@@ -2789,7 +2789,7 @@
         <v>3.56</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
     </row>
@@ -2821,7 +2821,7 @@
         <v>4.51</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
     </row>
@@ -2857,7 +2857,7 @@
         <v>15.02</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
     </row>
@@ -2893,7 +2893,7 @@
         <v>1237.96</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
     </row>
@@ -2929,7 +2929,7 @@
         <v>16.96</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
     </row>
@@ -2965,7 +2965,7 @@
         <v>88.43000000000001</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
     </row>
@@ -3001,7 +3001,7 @@
         <v>19.97</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
     </row>
@@ -3037,7 +3037,7 @@
         <v>206.33</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
     </row>
@@ -3073,7 +3073,7 @@
         <v>19.34</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
     </row>
@@ -3105,7 +3105,7 @@
         <v>63.48</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
     </row>
@@ -3141,7 +3141,7 @@
         <v>16.29</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
     </row>
@@ -3177,7 +3177,7 @@
         <v>13.99</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
     </row>
@@ -3213,7 +3213,7 @@
         <v>95.23</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
     </row>
@@ -3249,7 +3249,7 @@
         <v>8.6</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
     </row>
@@ -3285,7 +3285,7 @@
         <v>14.39</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
     </row>
@@ -3317,7 +3317,7 @@
         <v>11.52</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
     </row>
@@ -3353,7 +3353,7 @@
         <v>44.22</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
     </row>
@@ -3389,7 +3389,7 @@
         <v>19.35</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
     </row>
@@ -3425,7 +3425,7 @@
         <v>14.17</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J83" s="2" t="inlineStr"/>
     </row>
@@ -3461,7 +3461,7 @@
         <v>11.28</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
     </row>
@@ -3497,7 +3497,7 @@
         <v>13.81</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
     </row>
@@ -3533,7 +3533,7 @@
         <v>15.79</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
     </row>
@@ -3569,7 +3569,7 @@
         <v>27.62</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
     </row>
@@ -3601,7 +3601,7 @@
         <v>17.27</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
     </row>
@@ -3637,7 +3637,7 @@
         <v>1110</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
     </row>
@@ -3669,7 +3669,7 @@
         <v>1110</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
     </row>
@@ -3701,7 +3701,7 @@
         <v>1110</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J91" s="2" t="inlineStr"/>
     </row>
@@ -3737,7 +3737,7 @@
         <v>18.73</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
     </row>
@@ -3773,7 +3773,7 @@
         <v>12.14</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J93" s="2" t="inlineStr"/>
     </row>
@@ -3809,7 +3809,7 @@
         <v>8.630000000000001</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J94" s="2" t="inlineStr"/>
     </row>
@@ -3845,7 +3845,7 @@
         <v>6.42</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J95" s="2" t="inlineStr"/>
     </row>
@@ -3877,7 +3877,7 @@
         <v>10.83</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J96" s="2" t="inlineStr"/>
     </row>
@@ -3909,7 +3909,7 @@
         <v>9.57</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="J97" s="2" t="inlineStr"/>
     </row>
@@ -3945,7 +3945,7 @@
         <v>17.27</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
     </row>
@@ -3981,7 +3981,7 @@
         <v>11.51</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
     </row>
@@ -4017,7 +4017,7 @@
         <v>7.47</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J100" s="2" t="inlineStr"/>
     </row>
@@ -4053,7 +4053,7 @@
         <v>9.789999999999999</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J101" s="2" t="inlineStr"/>
     </row>
@@ -4089,7 +4089,7 @@
         <v>9.68</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J102" s="2" t="inlineStr"/>
     </row>
@@ -4125,7 +4125,7 @@
         <v>33.3</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J103" s="2" t="inlineStr"/>
     </row>
@@ -4157,7 +4157,7 @@
         <v>20.14</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
     </row>
@@ -4193,7 +4193,7 @@
         <v>11.62</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J105" s="2" t="inlineStr"/>
     </row>
@@ -4229,7 +4229,7 @@
         <v>23.56</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
     </row>
@@ -4265,7 +4265,7 @@
         <v>4.57</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J107" s="2" t="inlineStr"/>
     </row>
@@ -4297,7 +4297,7 @@
         <v>3.34</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J108" s="2" t="inlineStr"/>
     </row>
@@ -4333,7 +4333,7 @@
         <v>3.65</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="J109" s="2" t="inlineStr"/>
     </row>
@@ -4369,7 +4369,7 @@
         <v>364.86</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J110" s="2" t="inlineStr"/>
     </row>
@@ -4405,7 +4405,7 @@
         <v>10.73</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J111" s="2" t="inlineStr"/>
     </row>
@@ -4441,7 +4441,7 @@
         <v>23.8</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J112" s="2" t="inlineStr"/>
     </row>
@@ -4477,7 +4477,7 @@
         <v>10.52</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J113" s="2" t="inlineStr"/>
     </row>
@@ -4513,7 +4513,7 @@
         <v>19.55</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J114" s="2" t="inlineStr"/>
     </row>
@@ -4545,7 +4545,7 @@
         <v>9.69</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J115" s="2" t="inlineStr"/>
     </row>
@@ -4581,7 +4581,7 @@
         <v>20.27</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J116" s="2" t="inlineStr"/>
     </row>
@@ -4617,7 +4617,7 @@
         <v>13.51</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J117" s="2" t="inlineStr"/>
     </row>
@@ -4653,7 +4653,7 @@
         <v>6.57</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J118" s="2" t="inlineStr"/>
     </row>
@@ -4689,7 +4689,7 @@
         <v>19.55</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J119" s="2" t="inlineStr"/>
     </row>
@@ -4725,7 +4725,7 @@
         <v>16.58</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J120" s="2" t="inlineStr"/>
     </row>
@@ -4761,7 +4761,7 @@
         <v>6.95</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J121" s="2" t="inlineStr"/>
     </row>
@@ -4797,7 +4797,7 @@
         <v>11.52</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J122" s="2" t="inlineStr"/>
     </row>
@@ -4829,7 +4829,7 @@
         <v>20.27</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J123" s="2" t="inlineStr"/>
     </row>
@@ -4865,7 +4865,7 @@
         <v>136.82</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J124" s="2" t="inlineStr"/>
     </row>
@@ -4901,7 +4901,7 @@
         <v>12.73</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J125" s="2" t="inlineStr"/>
     </row>
@@ -4937,7 +4937,7 @@
         <v>7.26</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J126" s="2" t="inlineStr"/>
     </row>
@@ -4973,7 +4973,7 @@
         <v>6.26</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J127" s="2" t="inlineStr"/>
     </row>
@@ -5009,7 +5009,7 @@
         <v>5.13</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J128" s="2" t="inlineStr"/>
     </row>
@@ -5045,7 +5045,7 @@
         <v>3.19</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J129" s="2" t="inlineStr"/>
     </row>
@@ -5077,7 +5077,7 @@
         <v>2.86</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J130" s="2" t="inlineStr"/>
     </row>
@@ -5109,7 +5109,7 @@
         <v>3.25</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J131" s="2" t="inlineStr"/>
     </row>
@@ -5141,7 +5141,7 @@
         <v>26</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J132" s="2" t="inlineStr"/>
     </row>
@@ -5177,7 +5177,7 @@
         <v>19.5</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J133" s="2" t="inlineStr"/>
     </row>
@@ -5213,7 +5213,7 @@
         <v>877.5</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J134" s="2" t="inlineStr"/>
     </row>
@@ -5249,7 +5249,7 @@
         <v>100.29</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J135" s="2" t="inlineStr"/>
     </row>
@@ -5285,7 +5285,7 @@
         <v>15.13</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J136" s="2" t="inlineStr"/>
     </row>
@@ -5321,7 +5321,7 @@
         <v>33.43</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J137" s="2" t="inlineStr"/>
     </row>
@@ -5357,7 +5357,7 @@
         <v>9.970000000000001</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J138" s="2" t="inlineStr"/>
     </row>
@@ -5389,7 +5389,7 @@
         <v>12.9</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J139" s="2" t="inlineStr"/>
     </row>
@@ -5421,7 +5421,7 @@
         <v>28.08</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J140" s="2" t="inlineStr"/>
     </row>
@@ -5457,7 +5457,7 @@
         <v>17.12</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J141" s="2" t="inlineStr"/>
     </row>
@@ -5493,7 +5493,7 @@
         <v>14.94</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J142" s="2" t="inlineStr"/>
     </row>
@@ -5525,7 +5525,7 @@
         <v>1755</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J143" s="2" t="inlineStr"/>
     </row>
@@ -5557,7 +5557,7 @@
         <v>1755</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
     </row>
@@ -5589,7 +5589,7 @@
         <v>1755</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J145" s="2" t="inlineStr"/>
     </row>
@@ -5625,7 +5625,7 @@
         <v>6.46</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J146" s="2" t="inlineStr"/>
     </row>
@@ -5661,7 +5661,7 @@
         <v>6.31</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J147" s="2" t="inlineStr"/>
     </row>
@@ -5697,7 +5697,7 @@
         <v>14.94</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J148" s="2" t="inlineStr"/>
     </row>
@@ -5733,7 +5733,7 @@
         <v>4.78</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J149" s="2" t="inlineStr"/>
     </row>
@@ -5769,7 +5769,7 @@
         <v>5.9</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J150" s="2" t="inlineStr"/>
     </row>
@@ -5801,7 +5801,7 @@
         <v>1904.18</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J151" s="2" t="inlineStr"/>
     </row>
@@ -5837,7 +5837,7 @@
         <v>8.73</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J152" s="2" t="inlineStr"/>
     </row>
@@ -5873,7 +5873,7 @@
         <v>50.11</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J153" s="2" t="inlineStr"/>
     </row>
@@ -5909,7 +5909,7 @@
         <v>16.14</v>
       </c>
       <c r="I154" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J154" s="2" t="inlineStr"/>
     </row>
@@ -5945,7 +5945,7 @@
         <v>380.84</v>
       </c>
       <c r="I155" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J155" s="2" t="inlineStr"/>
     </row>
@@ -5981,7 +5981,7 @@
         <v>21.76</v>
       </c>
       <c r="I156" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J156" s="2" t="inlineStr"/>
     </row>
@@ -6017,7 +6017,7 @@
         <v>51.82</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J157" s="2" t="inlineStr"/>
     </row>
@@ -6049,7 +6049,7 @@
         <v>963.53</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J158" s="2" t="inlineStr"/>
     </row>
@@ -6085,7 +6085,7 @@
         <v>169.26</v>
       </c>
       <c r="I159" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J159" s="2" t="inlineStr"/>
     </row>
@@ -6121,7 +6121,7 @@
         <v>35.26</v>
       </c>
       <c r="I160" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J160" s="2" t="inlineStr"/>
     </row>
@@ -6153,7 +6153,7 @@
         <v>12.09</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J161" s="2" t="inlineStr"/>
     </row>
@@ -6189,7 +6189,7 @@
         <v>7.21</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J162" s="2" t="inlineStr"/>
     </row>
@@ -6225,7 +6225,7 @@
         <v>64.23</v>
       </c>
       <c r="I163" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J163" s="2" t="inlineStr"/>
     </row>
@@ -6261,7 +6261,7 @@
         <v>963.52</v>
       </c>
       <c r="I164" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J164" s="2" t="inlineStr"/>
     </row>
@@ -6293,7 +6293,7 @@
         <v>1927.03</v>
       </c>
       <c r="I165" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J165" s="2" t="inlineStr"/>
     </row>
@@ -6329,7 +6329,7 @@
         <v>17.27</v>
       </c>
       <c r="I166" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J166" s="2" t="inlineStr"/>
     </row>
@@ -6365,7 +6365,7 @@
         <v>9.460000000000001</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J167" s="2" t="inlineStr"/>
     </row>
@@ -6401,7 +6401,7 @@
         <v>7.42</v>
       </c>
       <c r="I168" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J168" s="2" t="inlineStr"/>
     </row>
@@ -6437,7 +6437,7 @@
         <v>6.06</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J169" s="2" t="inlineStr"/>
     </row>
@@ -6473,7 +6473,7 @@
         <v>3.66</v>
       </c>
       <c r="I170" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J170" s="2" t="inlineStr"/>
     </row>
@@ -6509,7 +6509,7 @@
         <v>9.92</v>
       </c>
       <c r="I171" s="2" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J171" s="2" t="inlineStr"/>
     </row>
@@ -6545,7 +6545,7 @@
         <v>3.41</v>
       </c>
       <c r="I172" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J172" s="2" t="inlineStr"/>
     </row>
@@ -6581,7 +6581,7 @@
         <v>4.4</v>
       </c>
       <c r="I173" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J173" s="2" t="inlineStr"/>
     </row>
@@ -6617,7 +6617,7 @@
         <v>603.11</v>
       </c>
       <c r="I174" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J174" s="2" t="inlineStr"/>
     </row>
@@ -6649,7 +6649,7 @@
         <v>9.24</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J175" s="2" t="inlineStr"/>
     </row>
@@ -6685,7 +6685,7 @@
         <v>16.05</v>
       </c>
       <c r="I176" s="2" t="n">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J176" s="2" t="inlineStr"/>
     </row>
@@ -6717,7 +6717,7 @@
         <v>32.11</v>
       </c>
       <c r="I177" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J177" s="2" t="inlineStr"/>
     </row>
@@ -6753,7 +6753,7 @@
         <v>8.710000000000001</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J178" s="2" t="inlineStr"/>
     </row>
@@ -6789,7 +6789,7 @@
         <v>10.17</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J179" s="2" t="inlineStr"/>
     </row>
@@ -6821,7 +6821,7 @@
         <v>16.05</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J180" s="2" t="inlineStr"/>
     </row>
@@ -6857,7 +6857,7 @@
         <v>7.82</v>
       </c>
       <c r="I181" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J181" s="2" t="inlineStr"/>
     </row>
@@ -6893,7 +6893,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="I182" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J182" s="2" t="inlineStr"/>
     </row>
@@ -6929,7 +6929,7 @@
         <v>5.26</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J183" s="2" t="inlineStr"/>
     </row>
@@ -6965,7 +6965,7 @@
         <v>19.06</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J184" s="2" t="inlineStr"/>
     </row>
@@ -7001,7 +7001,7 @@
         <v>26.52</v>
       </c>
       <c r="I185" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J185" s="2" t="inlineStr"/>
     </row>
@@ -7033,7 +7033,7 @@
         <v>13.86</v>
       </c>
       <c r="I186" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J186" s="2" t="inlineStr"/>
     </row>
@@ -7069,7 +7069,7 @@
         <v>3.63</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J187" s="2" t="inlineStr"/>
     </row>
@@ -7105,7 +7105,7 @@
         <v>7.37</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J188" s="2" t="inlineStr"/>
     </row>
@@ -7141,7 +7141,7 @@
         <v>7.92</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
     </row>
@@ -7177,7 +7177,7 @@
         <v>13.36</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J190" s="2" t="inlineStr"/>
     </row>
@@ -7213,7 +7213,7 @@
         <v>10.43</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J191" s="2" t="inlineStr"/>
     </row>
@@ -7249,7 +7249,7 @@
         <v>10.57</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J192" s="2" t="inlineStr"/>
     </row>
@@ -7285,7 +7285,7 @@
         <v>5.35</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
     </row>
@@ -7321,7 +7321,7 @@
         <v>5.38</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J194" s="2" t="inlineStr"/>
     </row>
@@ -7357,7 +7357,7 @@
         <v>4.63</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J195" s="2" t="inlineStr"/>
     </row>
@@ -7393,7 +7393,7 @@
         <v>2.85</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J196" s="2" t="inlineStr"/>
     </row>
@@ -7429,7 +7429,7 @@
         <v>2.78</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J197" s="2" t="inlineStr"/>
     </row>
@@ -7465,7 +7465,7 @@
         <v>4.52</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J198" s="2" t="inlineStr"/>
     </row>
@@ -7501,7 +7501,7 @@
         <v>5.19</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J199" s="2" t="inlineStr"/>
     </row>
@@ -7533,7 +7533,7 @@
         <v>4.92</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J200" s="2" t="inlineStr"/>
     </row>
@@ -7569,7 +7569,7 @@
         <v>6.49</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J201" s="2" t="inlineStr"/>
     </row>
@@ -7605,7 +7605,7 @@
         <v>6.91</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J202" s="2" t="inlineStr"/>
     </row>
@@ -7641,7 +7641,7 @@
         <v>7.23</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J203" s="2" t="inlineStr"/>
     </row>
@@ -7677,7 +7677,7 @@
         <v>14.98</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J204" s="2" t="inlineStr"/>
     </row>
@@ -7713,7 +7713,7 @@
         <v>37.75</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J205" s="2" t="inlineStr"/>
     </row>
@@ -7749,7 +7749,7 @@
         <v>20.97</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J206" s="2" t="inlineStr"/>
     </row>
@@ -7785,7 +7785,7 @@
         <v>12.38</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J207" s="2" t="inlineStr"/>
     </row>
@@ -7821,7 +7821,7 @@
         <v>10.21</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J208" s="2" t="inlineStr"/>
     </row>
@@ -7857,7 +7857,7 @@
         <v>11.85</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J209" s="2" t="inlineStr"/>
     </row>
@@ -7893,7 +7893,7 @@
         <v>14.13</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J210" s="2" t="inlineStr"/>
     </row>
@@ -7929,7 +7929,7 @@
         <v>17.98</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J211" s="2" t="inlineStr"/>
     </row>
@@ -7961,7 +7961,7 @@
         <v>6.65</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J212" s="2" t="inlineStr"/>
     </row>
@@ -7993,7 +7993,7 @@
         <v>5.57</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J213" s="2" t="inlineStr"/>
     </row>
@@ -8029,7 +8029,7 @@
         <v>6.32</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J214" s="2" t="inlineStr"/>
     </row>
@@ -8065,7 +8065,7 @@
         <v>5.4</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J215" s="2" t="inlineStr"/>
     </row>
@@ -8101,7 +8101,7 @@
         <v>10.86</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J216" s="2" t="inlineStr"/>
     </row>
@@ -8137,7 +8137,7 @@
         <v>41.94</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J217" s="2" t="inlineStr"/>
     </row>
@@ -8173,7 +8173,7 @@
         <v>3.14</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J218" s="2" t="inlineStr"/>
     </row>
@@ -8209,7 +8209,7 @@
         <v>4.35</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J219" s="2" t="inlineStr"/>
     </row>
@@ -8241,7 +8241,7 @@
         <v>1705.13</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J220" s="2" t="inlineStr"/>
     </row>
@@ -8277,7 +8277,7 @@
         <v>12.82</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J221" s="2" t="inlineStr"/>
     </row>
@@ -8309,7 +8309,7 @@
         <v>56.84</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J222" s="2" t="inlineStr"/>
     </row>
@@ -8345,7 +8345,7 @@
         <v>31.58</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J223" s="2" t="inlineStr"/>
     </row>
@@ -8381,7 +8381,7 @@
         <v>32.79</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J224" s="2" t="inlineStr"/>
     </row>
@@ -8417,7 +8417,7 @@
         <v>54.13</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="J225" s="2" t="inlineStr"/>
     </row>
@@ -8453,7 +8453,7 @@
         <v>28.9</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J226" s="2" t="inlineStr"/>
     </row>
@@ -8489,7 +8489,7 @@
         <v>21.86</v>
       </c>
       <c r="I227" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J227" s="2" t="inlineStr"/>
     </row>
@@ -8525,7 +8525,7 @@
         <v>6.45</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J228" s="2" t="inlineStr"/>
     </row>
@@ -8561,7 +8561,7 @@
         <v>341</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J229" s="2" t="inlineStr"/>
     </row>
@@ -8593,7 +8593,7 @@
         <v>568.33</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J230" s="2" t="inlineStr"/>
     </row>
@@ -8625,7 +8625,7 @@
         <v>1705</v>
       </c>
       <c r="I231" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J231" s="2" t="inlineStr"/>
     </row>
@@ -8661,7 +8661,7 @@
         <v>13.41</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J232" s="2" t="inlineStr"/>
     </row>
@@ -8697,7 +8697,7 @@
         <v>6.25</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J233" s="2" t="inlineStr"/>
     </row>
@@ -8733,7 +8733,7 @@
         <v>5.33</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J234" s="2" t="inlineStr"/>
     </row>
@@ -8769,7 +8769,7 @@
         <v>5.96</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J235" s="2" t="inlineStr"/>
     </row>
@@ -8805,7 +8805,7 @@
         <v>13.92</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J236" s="2" t="inlineStr"/>
     </row>
@@ -8841,7 +8841,7 @@
         <v>3.74</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J237" s="2" t="inlineStr"/>
     </row>
@@ -8877,7 +8877,7 @@
         <v>5.06</v>
       </c>
       <c r="I238" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J238" s="2" t="inlineStr"/>
     </row>
@@ -8909,7 +8909,7 @@
         <v>735</v>
       </c>
       <c r="I239" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J239" s="2" t="inlineStr"/>
     </row>
@@ -8945,7 +8945,7 @@
         <v>16.28</v>
       </c>
       <c r="I240" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J240" s="2" t="inlineStr"/>
     </row>
@@ -8977,7 +8977,7 @@
         <v>8.01</v>
       </c>
       <c r="I241" s="2" t="n">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="J241" s="2" t="inlineStr"/>
     </row>
@@ -9009,7 +9009,7 @@
         <v>13.56</v>
       </c>
       <c r="I242" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J242" s="2" t="inlineStr"/>
     </row>
@@ -9045,7 +9045,7 @@
         <v>14.65</v>
       </c>
       <c r="I243" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J243" s="2" t="inlineStr"/>
     </row>
@@ -9081,7 +9081,7 @@
         <v>25.26</v>
       </c>
       <c r="I244" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J244" s="2" t="inlineStr"/>
     </row>
@@ -9117,7 +9117,7 @@
         <v>33.3</v>
       </c>
       <c r="I245" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J245" s="2" t="inlineStr"/>
     </row>
@@ -9149,7 +9149,7 @@
         <v>5.47</v>
       </c>
       <c r="I246" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J246" s="2" t="inlineStr"/>
     </row>
@@ -9181,7 +9181,7 @@
         <v>6.91</v>
       </c>
       <c r="I247" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J247" s="2" t="inlineStr"/>
     </row>
@@ -9217,7 +9217,7 @@
         <v>5.69</v>
       </c>
       <c r="I248" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J248" s="2" t="inlineStr"/>
     </row>
@@ -9249,7 +9249,7 @@
         <v>3.94</v>
       </c>
       <c r="I249" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J249" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         <v>2.74</v>
       </c>
       <c r="I250" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J250" s="2" t="inlineStr"/>
     </row>
@@ -9317,7 +9317,7 @@
         <v>2.56</v>
       </c>
       <c r="I251" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J251" s="2" t="inlineStr"/>
     </row>
@@ -9353,7 +9353,7 @@
         <v>2.8</v>
       </c>
       <c r="I252" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J252" s="2" t="inlineStr"/>
     </row>
@@ -9389,7 +9389,7 @@
         <v>6.74</v>
       </c>
       <c r="I253" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J253" s="2" t="inlineStr"/>
     </row>
@@ -9425,7 +9425,7 @@
         <v>3.7</v>
       </c>
       <c r="I254" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J254" s="2" t="inlineStr"/>
     </row>
@@ -9461,7 +9461,7 @@
         <v>11.49</v>
       </c>
       <c r="I255" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J255" s="2" t="inlineStr"/>
     </row>
@@ -9497,7 +9497,7 @@
         <v>7.46</v>
       </c>
       <c r="I256" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J256" s="2" t="inlineStr"/>
     </row>
@@ -9533,7 +9533,7 @@
         <v>28.08</v>
       </c>
       <c r="I257" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J257" s="2" t="inlineStr"/>
     </row>
@@ -9569,7 +9569,7 @@
         <v>13.07</v>
       </c>
       <c r="I258" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J258" s="2" t="inlineStr"/>
     </row>
@@ -9605,7 +9605,7 @@
         <v>11.66</v>
       </c>
       <c r="I259" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J259" s="2" t="inlineStr"/>
     </row>
@@ -9641,7 +9641,7 @@
         <v>6.61</v>
       </c>
       <c r="I260" s="2" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J260" s="2" t="inlineStr"/>
     </row>
@@ -9677,7 +9677,7 @@
         <v>3.09</v>
       </c>
       <c r="I261" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J261" s="2" t="inlineStr"/>
     </row>
@@ -9713,7 +9713,7 @@
         <v>3.35</v>
       </c>
       <c r="I262" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J262" s="2" t="inlineStr"/>
     </row>
@@ -9749,7 +9749,7 @@
         <v>35.84</v>
       </c>
       <c r="I263" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J263" s="2" t="inlineStr"/>
     </row>
@@ -9785,7 +9785,7 @@
         <v>13.59</v>
       </c>
       <c r="I264" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J264" s="2" t="inlineStr"/>
     </row>
@@ -9817,7 +9817,7 @@
         <v>523.84</v>
       </c>
       <c r="I265" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J265" s="2" t="inlineStr"/>
     </row>
@@ -9853,7 +9853,7 @@
         <v>16.06</v>
       </c>
       <c r="I266" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J266" s="2" t="inlineStr"/>
     </row>
@@ -9885,7 +9885,7 @@
         <v>12.46</v>
       </c>
       <c r="I267" s="2" t="n">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="J267" s="2" t="inlineStr"/>
     </row>
@@ -9921,7 +9921,7 @@
         <v>23.36</v>
       </c>
       <c r="I268" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J268" s="2" t="inlineStr"/>
     </row>
@@ -9957,7 +9957,7 @@
         <v>4.3</v>
       </c>
       <c r="I269" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J269" s="2" t="inlineStr"/>
     </row>
@@ -9993,7 +9993,7 @@
         <v>5.84</v>
       </c>
       <c r="I270" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J270" s="2" t="inlineStr"/>
     </row>
@@ -10029,7 +10029,7 @@
         <v>1.84</v>
       </c>
       <c r="I271" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J271" s="2" t="inlineStr"/>
     </row>
@@ -10065,7 +10065,7 @@
         <v>1.97</v>
       </c>
       <c r="I272" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J272" s="2" t="inlineStr"/>
     </row>
@@ -10101,7 +10101,7 @@
         <v>8.81</v>
       </c>
       <c r="I273" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J273" s="2" t="inlineStr"/>
     </row>
@@ -10137,7 +10137,7 @@
         <v>7.52</v>
       </c>
       <c r="I274" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J274" s="2" t="inlineStr"/>
     </row>
@@ -10173,7 +10173,7 @@
         <v>6.41</v>
       </c>
       <c r="I275" s="2" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J275" s="2" t="inlineStr"/>
     </row>
@@ -10209,7 +10209,7 @@
         <v>24.58</v>
       </c>
       <c r="I276" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J276" s="2" t="inlineStr"/>
     </row>
@@ -10245,7 +10245,7 @@
         <v>16.86</v>
       </c>
       <c r="I277" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J277" s="2" t="inlineStr"/>
     </row>
@@ -10281,7 +10281,7 @@
         <v>4.99</v>
       </c>
       <c r="I278" s="2" t="n">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J278" s="2" t="inlineStr"/>
     </row>
@@ -10317,7 +10317,7 @@
         <v>2.83</v>
       </c>
       <c r="I279" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J279" s="2" t="inlineStr"/>
     </row>
@@ -10353,7 +10353,7 @@
         <v>3.16</v>
       </c>
       <c r="I280" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J280" s="2" t="inlineStr"/>
     </row>
@@ -10385,7 +10385,7 @@
         <v>32.51</v>
       </c>
       <c r="I281" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="J281" s="2" t="inlineStr"/>
     </row>
@@ -10421,7 +10421,7 @@
         <v>17.67</v>
       </c>
       <c r="I282" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J282" s="2" t="inlineStr"/>
     </row>
@@ -10457,7 +10457,7 @@
         <v>23.9</v>
       </c>
       <c r="I283" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J283" s="2" t="inlineStr"/>
     </row>
@@ -10493,7 +10493,7 @@
         <v>5</v>
       </c>
       <c r="I284" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J284" s="2" t="inlineStr"/>
     </row>
@@ -10529,7 +10529,7 @@
         <v>7.02</v>
       </c>
       <c r="I285" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J285" s="2" t="inlineStr"/>
     </row>
@@ -10565,7 +10565,7 @@
         <v>6.79</v>
       </c>
       <c r="I286" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J286" s="2" t="inlineStr"/>
     </row>
@@ -10601,7 +10601,7 @@
         <v>12.02</v>
       </c>
       <c r="I287" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J287" s="2" t="inlineStr"/>
     </row>
@@ -10637,7 +10637,7 @@
         <v>9.57</v>
       </c>
       <c r="I288" s="2" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J288" s="2" t="inlineStr"/>
     </row>
@@ -10673,7 +10673,7 @@
         <v>13.74</v>
       </c>
       <c r="I289" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J289" s="2" t="inlineStr"/>
     </row>
@@ -10705,7 +10705,7 @@
         <v>6.7</v>
       </c>
       <c r="I290" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J290" s="2" t="inlineStr"/>
     </row>
@@ -10741,7 +10741,7 @@
         <v>11.28</v>
       </c>
       <c r="I291" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J291" s="2" t="inlineStr"/>
     </row>
@@ -10777,7 +10777,7 @@
         <v>24.72</v>
       </c>
       <c r="I292" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J292" s="2" t="inlineStr"/>
     </row>
@@ -10813,7 +10813,7 @@
         <v>16.07</v>
       </c>
       <c r="I293" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J293" s="2" t="inlineStr"/>
     </row>
@@ -10849,7 +10849,7 @@
         <v>8.27</v>
       </c>
       <c r="I294" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J294" s="2" t="inlineStr"/>
     </row>
@@ -10885,7 +10885,7 @@
         <v>11.24</v>
       </c>
       <c r="I295" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J295" s="2" t="inlineStr"/>
     </row>
@@ -10921,7 +10921,7 @@
         <v>17.36</v>
       </c>
       <c r="I296" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J296" s="2" t="inlineStr"/>
     </row>
@@ -10957,7 +10957,7 @@
         <v>6.59</v>
       </c>
       <c r="I297" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J297" s="2" t="inlineStr"/>
     </row>
@@ -10989,7 +10989,7 @@
         <v>5.44</v>
       </c>
       <c r="I298" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J298" s="2" t="inlineStr"/>
     </row>
@@ -11025,7 +11025,7 @@
         <v>3.79</v>
       </c>
       <c r="I299" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J299" s="2" t="inlineStr"/>
     </row>
@@ -11061,7 +11061,7 @@
         <v>8.42</v>
       </c>
       <c r="I300" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J300" s="2" t="inlineStr"/>
     </row>
@@ -11097,7 +11097,7 @@
         <v>27.74</v>
       </c>
       <c r="I301" s="2" t="n">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J301" s="2" t="inlineStr"/>
     </row>
@@ -11133,7 +11133,7 @@
         <v>30.75</v>
       </c>
       <c r="I302" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J302" s="2" t="inlineStr"/>
     </row>
@@ -11169,7 +11169,7 @@
         <v>11.99</v>
       </c>
       <c r="I303" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J303" s="2" t="inlineStr"/>
     </row>
@@ -11205,7 +11205,7 @@
         <v>56.59</v>
       </c>
       <c r="I304" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="J304" s="2" t="inlineStr"/>
     </row>
@@ -11241,7 +11241,7 @@
         <v>14.15</v>
       </c>
       <c r="I305" s="2" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="J305" s="2" t="inlineStr"/>
     </row>
@@ -11277,7 +11277,7 @@
         <v>34.5</v>
       </c>
       <c r="I306" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J306" s="2" t="inlineStr"/>
     </row>
@@ -11313,7 +11313,7 @@
         <v>18.61</v>
       </c>
       <c r="I307" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J307" s="2" t="inlineStr"/>
     </row>
@@ -11349,7 +11349,7 @@
         <v>5.66</v>
       </c>
       <c r="I308" s="2" t="n">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="J308" s="2" t="inlineStr"/>
     </row>
@@ -11385,7 +11385,7 @@
         <v>15.72</v>
       </c>
       <c r="I309" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="J309" s="2" t="inlineStr"/>
     </row>
@@ -11421,7 +11421,7 @@
         <v>7.72</v>
       </c>
       <c r="I310" s="2" t="n">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="J310" s="2" t="inlineStr"/>
     </row>
@@ -11457,7 +11457,7 @@
         <v>19.86</v>
       </c>
       <c r="I311" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J311" s="2" t="inlineStr"/>
     </row>
@@ -11493,7 +11493,7 @@
         <v>13.56</v>
       </c>
       <c r="I312" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J312" s="2" t="inlineStr"/>
     </row>
@@ -11529,7 +11529,7 @@
         <v>10.3</v>
       </c>
       <c r="I313" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J313" s="2" t="inlineStr"/>
     </row>
@@ -11565,7 +11565,7 @@
         <v>17.16</v>
       </c>
       <c r="I314" s="2" t="n">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J314" s="2" t="inlineStr"/>
     </row>
@@ -11601,7 +11601,7 @@
         <v>6.47</v>
       </c>
       <c r="I315" s="2" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="J315" s="2" t="inlineStr"/>
     </row>
@@ -11637,7 +11637,7 @@
         <v>5.52</v>
       </c>
       <c r="I316" s="2" t="n">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="J316" s="2" t="inlineStr"/>
     </row>
@@ -11673,7 +11673,7 @@
         <v>5.25</v>
       </c>
       <c r="I317" s="2" t="n">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="J317" s="2" t="inlineStr"/>
     </row>
@@ -11709,7 +11709,7 @@
         <v>11.44</v>
       </c>
       <c r="I318" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J318" s="2" t="inlineStr"/>
     </row>
@@ -11745,7 +11745,7 @@
         <v>10.53</v>
       </c>
       <c r="I319" s="2" t="n">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="J319" s="2" t="inlineStr"/>
     </row>
@@ -11781,7 +11781,7 @@
         <v>16.95</v>
       </c>
       <c r="I320" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J320" s="2" t="inlineStr"/>
     </row>
@@ -11813,7 +11813,7 @@
         <v>3.28</v>
       </c>
       <c r="I321" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J321" s="2" t="inlineStr"/>
     </row>
@@ -11849,7 +11849,7 @@
         <v>4.06</v>
       </c>
       <c r="I322" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J322" s="2" t="inlineStr"/>
     </row>
@@ -11881,7 +11881,7 @@
         <v>42.23</v>
       </c>
       <c r="I323" s="2" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="J323" s="2" t="inlineStr"/>
     </row>
@@ -11913,7 +11913,7 @@
         <v>24.13</v>
       </c>
       <c r="I324" s="2" t="n">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J324" s="2" t="inlineStr"/>
     </row>
@@ -11949,7 +11949,7 @@
         <v>7.57</v>
       </c>
       <c r="I325" s="2" t="n">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="J325" s="2" t="inlineStr"/>
     </row>
@@ -11985,7 +11985,7 @@
         <v>11.5</v>
       </c>
       <c r="I326" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J326" s="2" t="inlineStr"/>
     </row>
@@ -12017,7 +12017,7 @@
         <v>14.61</v>
       </c>
       <c r="I327" s="2" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="J327" s="2" t="inlineStr"/>
     </row>
@@ -12053,7 +12053,7 @@
         <v>3.47</v>
       </c>
       <c r="I328" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J328" s="2" t="inlineStr"/>
     </row>
@@ -12089,7 +12089,7 @@
         <v>5.32</v>
       </c>
       <c r="I329" s="2" t="n">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="J329" s="2" t="inlineStr"/>
     </row>

</xml_diff>

<commit_message>
Update CW data 2026-09-01
</commit_message>
<xml_diff>
--- a/docs/downloads/KetQuaGiaoDich_latest.xlsx
+++ b/docs/downloads/KetQuaGiaoDich_latest.xlsx
@@ -573,7 +573,7 @@
         <v>8.06</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J2" s="2" t="inlineStr"/>
     </row>
@@ -609,7 +609,7 @@
         <v>328.36</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J3" s="2" t="inlineStr"/>
     </row>
@@ -645,7 +645,7 @@
         <v>18.76</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
     </row>
@@ -677,7 +677,7 @@
         <v>38.63</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J5" s="2" t="inlineStr"/>
     </row>
@@ -713,7 +713,7 @@
         <v>16.84</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J6" s="2" t="inlineStr"/>
     </row>
@@ -749,7 +749,7 @@
         <v>29.19</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J7" s="2" t="inlineStr"/>
     </row>
@@ -785,7 +785,7 @@
         <v>11.32</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J8" s="2" t="inlineStr"/>
     </row>
@@ -821,7 +821,7 @@
         <v>12.51</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J9" s="2" t="inlineStr"/>
     </row>
@@ -857,7 +857,7 @@
         <v>7.91</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J10" s="2" t="inlineStr"/>
     </row>
@@ -893,7 +893,7 @@
         <v>8.01</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J11" s="2" t="inlineStr"/>
     </row>
@@ -929,7 +929,7 @@
         <v>10.18</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J12" s="2" t="inlineStr"/>
     </row>
@@ -961,7 +961,7 @@
         <v>21.02</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J13" s="2" t="inlineStr"/>
     </row>
@@ -993,7 +993,7 @@
         <v>20.21</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J14" s="2" t="inlineStr"/>
     </row>
@@ -1025,7 +1025,7 @@
         <v>13.83</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J15" s="2" t="inlineStr"/>
     </row>
@@ -1061,7 +1061,7 @@
         <v>27.37</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" s="2" t="inlineStr"/>
     </row>
@@ -1097,7 +1097,7 @@
         <v>437.98</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J17" s="2" t="inlineStr"/>
     </row>
@@ -1129,7 +1129,7 @@
         <v>12.65</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J18" s="2" t="inlineStr"/>
     </row>
@@ -1161,7 +1161,7 @@
         <v>6.15</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J19" s="2" t="inlineStr"/>
     </row>
@@ -1197,7 +1197,7 @@
         <v>11.8</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J20" s="2" t="inlineStr"/>
     </row>
@@ -1233,7 +1233,7 @@
         <v>12.72</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J21" s="2" t="inlineStr"/>
     </row>
@@ -1269,7 +1269,7 @@
         <v>10.89</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J22" s="2" t="inlineStr"/>
     </row>
@@ -1301,7 +1301,7 @@
         <v>850.29</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J23" s="2" t="inlineStr"/>
     </row>
@@ -1337,7 +1337,7 @@
         <v>462.26</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J24" s="2" t="inlineStr"/>
     </row>
@@ -1373,7 +1373,7 @@
         <v>23.71</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J25" s="2" t="inlineStr"/>
     </row>
@@ -1409,7 +1409,7 @@
         <v>205.45</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J26" s="2" t="inlineStr"/>
     </row>
@@ -1445,7 +1445,7 @@
         <v>30.82</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J27" s="2" t="inlineStr"/>
     </row>
@@ -1481,7 +1481,7 @@
         <v>371.04</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J28" s="2" t="inlineStr"/>
     </row>
@@ -1513,7 +1513,7 @@
         <v>37.1</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J29" s="2" t="inlineStr"/>
     </row>
@@ -1549,7 +1549,7 @@
         <v>29.68</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J30" s="2" t="inlineStr"/>
     </row>
@@ -1581,7 +1581,7 @@
         <v>371.04</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
     </row>
@@ -1613,7 +1613,7 @@
         <v>742.08</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
     </row>
@@ -1645,7 +1645,7 @@
         <v>23.19</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J33" s="2" t="inlineStr"/>
     </row>
@@ -1681,7 +1681,7 @@
         <v>16.27</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J34" s="2" t="inlineStr"/>
     </row>
@@ -1717,7 +1717,7 @@
         <v>5.9</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J35" s="2" t="inlineStr"/>
     </row>
@@ -1753,7 +1753,7 @@
         <v>6.12</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J36" s="2" t="inlineStr"/>
     </row>
@@ -1789,7 +1789,7 @@
         <v>19.26</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J37" s="2" t="inlineStr"/>
     </row>
@@ -1825,7 +1825,7 @@
         <v>11.26</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J38" s="2" t="inlineStr"/>
     </row>
@@ -1861,7 +1861,7 @@
         <v>7.21</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
     </row>
@@ -1897,7 +1897,7 @@
         <v>12.04</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
     </row>
@@ -1933,7 +1933,7 @@
         <v>10.64</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J41" s="2" t="inlineStr"/>
     </row>
@@ -1969,7 +1969,7 @@
         <v>25.79</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J42" s="2" t="inlineStr"/>
     </row>
@@ -2005,7 +2005,7 @@
         <v>75.20999999999999</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" s="2" t="inlineStr"/>
     </row>
@@ -2037,7 +2037,7 @@
         <v>902.5</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" s="2" t="inlineStr"/>
     </row>
@@ -2073,7 +2073,7 @@
         <v>7.97</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J45" s="2" t="inlineStr"/>
     </row>
@@ -2109,7 +2109,7 @@
         <v>6.78</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J46" s="2" t="inlineStr"/>
     </row>
@@ -2145,7 +2145,7 @@
         <v>6.78</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J47" s="2" t="inlineStr"/>
     </row>
@@ -2181,7 +2181,7 @@
         <v>5.4</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J48" s="2" t="inlineStr"/>
     </row>
@@ -2217,7 +2217,7 @@
         <v>9.890000000000001</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J49" s="2" t="inlineStr"/>
     </row>
@@ -2253,7 +2253,7 @@
         <v>7.47</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J50" s="2" t="inlineStr"/>
     </row>
@@ -2289,7 +2289,7 @@
         <v>4.09</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
     </row>
@@ -2325,7 +2325,7 @@
         <v>4.52</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
     </row>
@@ -2361,7 +2361,7 @@
         <v>30.05</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
     </row>
@@ -2397,7 +2397,7 @@
         <v>6.43</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
     </row>
@@ -2433,7 +2433,7 @@
         <v>29.89</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J55" s="2" t="inlineStr"/>
     </row>
@@ -2469,7 +2469,7 @@
         <v>5.19</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
     </row>
@@ -2505,7 +2505,7 @@
         <v>12.69</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
     </row>
@@ -2541,7 +2541,7 @@
         <v>9</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J58" s="2" t="inlineStr"/>
     </row>
@@ -2577,7 +2577,7 @@
         <v>18.53</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J59" s="2" t="inlineStr"/>
     </row>
@@ -2613,7 +2613,7 @@
         <v>10.22</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
     </row>
@@ -2649,7 +2649,7 @@
         <v>4.79</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
     </row>
@@ -2685,7 +2685,7 @@
         <v>3.34</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
     </row>
@@ -2717,7 +2717,7 @@
         <v>10.18</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J63" s="2" t="inlineStr"/>
     </row>
@@ -2753,7 +2753,7 @@
         <v>8.42</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J64" s="2" t="inlineStr"/>
     </row>
@@ -2789,7 +2789,7 @@
         <v>3.56</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J65" s="2" t="inlineStr"/>
     </row>
@@ -2821,7 +2821,7 @@
         <v>4.51</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J66" s="2" t="inlineStr"/>
     </row>
@@ -2857,7 +2857,7 @@
         <v>15.02</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J67" s="2" t="inlineStr"/>
     </row>
@@ -2893,7 +2893,7 @@
         <v>1237.96</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J68" s="2" t="inlineStr"/>
     </row>
@@ -2929,7 +2929,7 @@
         <v>16.96</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J69" s="2" t="inlineStr"/>
     </row>
@@ -2965,7 +2965,7 @@
         <v>88.43000000000001</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
     </row>
@@ -3001,7 +3001,7 @@
         <v>19.97</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J71" s="2" t="inlineStr"/>
     </row>
@@ -3037,7 +3037,7 @@
         <v>206.33</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
     </row>
@@ -3073,7 +3073,7 @@
         <v>19.34</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
     </row>
@@ -3105,7 +3105,7 @@
         <v>63.48</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
     </row>
@@ -3141,7 +3141,7 @@
         <v>16.29</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
     </row>
@@ -3177,7 +3177,7 @@
         <v>13.99</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
     </row>
@@ -3213,7 +3213,7 @@
         <v>95.23</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J77" s="2" t="inlineStr"/>
     </row>
@@ -3249,7 +3249,7 @@
         <v>8.6</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J78" s="2" t="inlineStr"/>
     </row>
@@ -3285,7 +3285,7 @@
         <v>14.39</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="J79" s="2" t="inlineStr"/>
     </row>
@@ -3317,7 +3317,7 @@
         <v>11.52</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J80" s="2" t="inlineStr"/>
     </row>
@@ -3353,7 +3353,7 @@
         <v>44.22</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J81" s="2" t="inlineStr"/>
     </row>
@@ -3389,7 +3389,7 @@
         <v>19.35</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J82" s="2" t="inlineStr"/>
     </row>
@@ -3425,7 +3425,7 @@
         <v>14.17</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J83" s="2" t="inlineStr"/>
     </row>
@@ -3461,7 +3461,7 @@
         <v>11.28</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J84" s="2" t="inlineStr"/>
     </row>
@@ -3497,7 +3497,7 @@
         <v>13.81</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J85" s="2" t="inlineStr"/>
     </row>
@@ -3533,7 +3533,7 @@
         <v>15.79</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J86" s="2" t="inlineStr"/>
     </row>
@@ -3569,7 +3569,7 @@
         <v>27.62</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J87" s="2" t="inlineStr"/>
     </row>
@@ -3601,7 +3601,7 @@
         <v>17.27</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J88" s="2" t="inlineStr"/>
     </row>
@@ -3637,7 +3637,7 @@
         <v>1110</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J89" s="2" t="inlineStr"/>
     </row>
@@ -3669,7 +3669,7 @@
         <v>1110</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J90" s="2" t="inlineStr"/>
     </row>
@@ -3701,7 +3701,7 @@
         <v>1110</v>
       </c>
       <c r="I91" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J91" s="2" t="inlineStr"/>
     </row>
@@ -3737,7 +3737,7 @@
         <v>18.73</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J92" s="2" t="inlineStr"/>
     </row>
@@ -3773,7 +3773,7 @@
         <v>12.14</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J93" s="2" t="inlineStr"/>
     </row>
@@ -3809,7 +3809,7 @@
         <v>8.630000000000001</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J94" s="2" t="inlineStr"/>
     </row>
@@ -3845,7 +3845,7 @@
         <v>6.42</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J95" s="2" t="inlineStr"/>
     </row>
@@ -3877,7 +3877,7 @@
         <v>10.83</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J96" s="2" t="inlineStr"/>
     </row>
@@ -3909,7 +3909,7 @@
         <v>9.57</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J97" s="2" t="inlineStr"/>
     </row>
@@ -3945,7 +3945,7 @@
         <v>17.27</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J98" s="2" t="inlineStr"/>
     </row>
@@ -3981,7 +3981,7 @@
         <v>11.51</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J99" s="2" t="inlineStr"/>
     </row>
@@ -4017,7 +4017,7 @@
         <v>7.47</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J100" s="2" t="inlineStr"/>
     </row>
@@ -4053,7 +4053,7 @@
         <v>9.789999999999999</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J101" s="2" t="inlineStr"/>
     </row>
@@ -4089,7 +4089,7 @@
         <v>9.68</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J102" s="2" t="inlineStr"/>
     </row>
@@ -4125,7 +4125,7 @@
         <v>33.3</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J103" s="2" t="inlineStr"/>
     </row>
@@ -4157,7 +4157,7 @@
         <v>20.14</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J104" s="2" t="inlineStr"/>
     </row>
@@ -4193,7 +4193,7 @@
         <v>11.62</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J105" s="2" t="inlineStr"/>
     </row>
@@ -4229,7 +4229,7 @@
         <v>23.56</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J106" s="2" t="inlineStr"/>
     </row>
@@ -4265,7 +4265,7 @@
         <v>4.57</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J107" s="2" t="inlineStr"/>
     </row>
@@ -4297,7 +4297,7 @@
         <v>3.34</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J108" s="2" t="inlineStr"/>
     </row>
@@ -4333,7 +4333,7 @@
         <v>3.65</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J109" s="2" t="inlineStr"/>
     </row>
@@ -4369,7 +4369,7 @@
         <v>364.86</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J110" s="2" t="inlineStr"/>
     </row>
@@ -4405,7 +4405,7 @@
         <v>10.73</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J111" s="2" t="inlineStr"/>
     </row>
@@ -4441,7 +4441,7 @@
         <v>23.8</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J112" s="2" t="inlineStr"/>
     </row>
@@ -4477,7 +4477,7 @@
         <v>10.52</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J113" s="2" t="inlineStr"/>
     </row>
@@ -4513,7 +4513,7 @@
         <v>19.55</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J114" s="2" t="inlineStr"/>
     </row>
@@ -4545,7 +4545,7 @@
         <v>9.69</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J115" s="2" t="inlineStr"/>
     </row>
@@ -4581,7 +4581,7 @@
         <v>20.27</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J116" s="2" t="inlineStr"/>
     </row>
@@ -4617,7 +4617,7 @@
         <v>13.51</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J117" s="2" t="inlineStr"/>
     </row>
@@ -4653,7 +4653,7 @@
         <v>6.57</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J118" s="2" t="inlineStr"/>
     </row>
@@ -4689,7 +4689,7 @@
         <v>19.55</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J119" s="2" t="inlineStr"/>
     </row>
@@ -4725,7 +4725,7 @@
         <v>16.58</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J120" s="2" t="inlineStr"/>
     </row>
@@ -4761,7 +4761,7 @@
         <v>6.95</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J121" s="2" t="inlineStr"/>
     </row>
@@ -4797,7 +4797,7 @@
         <v>11.52</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J122" s="2" t="inlineStr"/>
     </row>
@@ -4829,7 +4829,7 @@
         <v>20.27</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J123" s="2" t="inlineStr"/>
     </row>
@@ -4865,7 +4865,7 @@
         <v>136.82</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J124" s="2" t="inlineStr"/>
     </row>
@@ -4901,7 +4901,7 @@
         <v>12.73</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J125" s="2" t="inlineStr"/>
     </row>
@@ -4937,7 +4937,7 @@
         <v>7.26</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J126" s="2" t="inlineStr"/>
     </row>
@@ -4973,7 +4973,7 @@
         <v>6.26</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J127" s="2" t="inlineStr"/>
     </row>
@@ -5009,7 +5009,7 @@
         <v>5.13</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J128" s="2" t="inlineStr"/>
     </row>
@@ -5045,7 +5045,7 @@
         <v>3.19</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J129" s="2" t="inlineStr"/>
     </row>
@@ -5077,7 +5077,7 @@
         <v>2.86</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J130" s="2" t="inlineStr"/>
     </row>
@@ -5109,7 +5109,7 @@
         <v>3.25</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J131" s="2" t="inlineStr"/>
     </row>
@@ -5141,7 +5141,7 @@
         <v>26</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J132" s="2" t="inlineStr"/>
     </row>
@@ -5177,7 +5177,7 @@
         <v>19.5</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J133" s="2" t="inlineStr"/>
     </row>
@@ -5213,7 +5213,7 @@
         <v>877.5</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J134" s="2" t="inlineStr"/>
     </row>
@@ -5249,7 +5249,7 @@
         <v>100.29</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J135" s="2" t="inlineStr"/>
     </row>
@@ -5285,7 +5285,7 @@
         <v>15.13</v>
       </c>
       <c r="I136" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J136" s="2" t="inlineStr"/>
     </row>
@@ -5321,7 +5321,7 @@
         <v>33.43</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J137" s="2" t="inlineStr"/>
     </row>
@@ -5357,7 +5357,7 @@
         <v>9.970000000000001</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J138" s="2" t="inlineStr"/>
     </row>
@@ -5389,7 +5389,7 @@
         <v>12.9</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J139" s="2" t="inlineStr"/>
     </row>
@@ -5421,7 +5421,7 @@
         <v>28.08</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J140" s="2" t="inlineStr"/>
     </row>
@@ -5457,7 +5457,7 @@
         <v>17.12</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J141" s="2" t="inlineStr"/>
     </row>
@@ -5493,7 +5493,7 @@
         <v>14.94</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J142" s="2" t="inlineStr"/>
     </row>
@@ -5525,7 +5525,7 @@
         <v>1755</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J143" s="2" t="inlineStr"/>
     </row>
@@ -5557,7 +5557,7 @@
         <v>1755</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
     </row>
@@ -5589,7 +5589,7 @@
         <v>1755</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J145" s="2" t="inlineStr"/>
     </row>
@@ -5625,7 +5625,7 @@
         <v>6.46</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J146" s="2" t="inlineStr"/>
     </row>
@@ -5661,7 +5661,7 @@
         <v>6.31</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J147" s="2" t="inlineStr"/>
     </row>
@@ -5697,7 +5697,7 @@
         <v>14.94</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J148" s="2" t="inlineStr"/>
     </row>
@@ -5733,7 +5733,7 @@
         <v>4.78</v>
       </c>
       <c r="I149" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J149" s="2" t="inlineStr"/>
     </row>
@@ -5769,7 +5769,7 @@
         <v>5.9</v>
       </c>
       <c r="I150" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J150" s="2" t="inlineStr"/>
     </row>
@@ -5801,7 +5801,7 @@
         <v>1904.18</v>
       </c>
       <c r="I151" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J151" s="2" t="inlineStr"/>
     </row>
@@ -5837,7 +5837,7 @@
         <v>8.73</v>
       </c>
       <c r="I152" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J152" s="2" t="inlineStr"/>
     </row>
@@ -5873,7 +5873,7 @@
         <v>50.11</v>
       </c>
       <c r="I153" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J153" s="2" t="inlineStr"/>
     </row>
@@ -5909,7 +5909,7 @@
         <v>16.14</v>
       </c>
       <c r="I154" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J154" s="2" t="inlineStr"/>
     </row>
@@ -5945,7 +5945,7 @@
         <v>380.84</v>
       </c>
       <c r="I155" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J155" s="2" t="inlineStr"/>
     </row>
@@ -5981,7 +5981,7 @@
         <v>21.76</v>
       </c>
       <c r="I156" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J156" s="2" t="inlineStr"/>
     </row>
@@ -6017,7 +6017,7 @@
         <v>51.82</v>
       </c>
       <c r="I157" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J157" s="2" t="inlineStr"/>
     </row>
@@ -6049,7 +6049,7 @@
         <v>963.53</v>
       </c>
       <c r="I158" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J158" s="2" t="inlineStr"/>
     </row>
@@ -6085,7 +6085,7 @@
         <v>169.26</v>
       </c>
       <c r="I159" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J159" s="2" t="inlineStr"/>
     </row>
@@ -6121,7 +6121,7 @@
         <v>35.26</v>
       </c>
       <c r="I160" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J160" s="2" t="inlineStr"/>
     </row>
@@ -6153,7 +6153,7 @@
         <v>12.09</v>
       </c>
       <c r="I161" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J161" s="2" t="inlineStr"/>
     </row>
@@ -6189,7 +6189,7 @@
         <v>7.21</v>
       </c>
       <c r="I162" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J162" s="2" t="inlineStr"/>
     </row>
@@ -6225,7 +6225,7 @@
         <v>64.23</v>
       </c>
       <c r="I163" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J163" s="2" t="inlineStr"/>
     </row>
@@ -6261,7 +6261,7 @@
         <v>963.52</v>
       </c>
       <c r="I164" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J164" s="2" t="inlineStr"/>
     </row>
@@ -6293,7 +6293,7 @@
         <v>1927.03</v>
       </c>
       <c r="I165" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J165" s="2" t="inlineStr"/>
     </row>
@@ -6329,7 +6329,7 @@
         <v>17.27</v>
       </c>
       <c r="I166" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J166" s="2" t="inlineStr"/>
     </row>
@@ -6365,7 +6365,7 @@
         <v>9.460000000000001</v>
       </c>
       <c r="I167" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J167" s="2" t="inlineStr"/>
     </row>
@@ -6401,7 +6401,7 @@
         <v>7.42</v>
       </c>
       <c r="I168" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J168" s="2" t="inlineStr"/>
     </row>
@@ -6437,7 +6437,7 @@
         <v>6.06</v>
       </c>
       <c r="I169" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J169" s="2" t="inlineStr"/>
     </row>
@@ -6473,7 +6473,7 @@
         <v>3.66</v>
       </c>
       <c r="I170" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J170" s="2" t="inlineStr"/>
     </row>
@@ -6509,7 +6509,7 @@
         <v>9.92</v>
       </c>
       <c r="I171" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J171" s="2" t="inlineStr"/>
     </row>
@@ -6545,7 +6545,7 @@
         <v>3.41</v>
       </c>
       <c r="I172" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J172" s="2" t="inlineStr"/>
     </row>
@@ -6581,7 +6581,7 @@
         <v>4.4</v>
       </c>
       <c r="I173" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J173" s="2" t="inlineStr"/>
     </row>
@@ -6617,7 +6617,7 @@
         <v>603.11</v>
       </c>
       <c r="I174" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J174" s="2" t="inlineStr"/>
     </row>
@@ -6649,7 +6649,7 @@
         <v>9.24</v>
       </c>
       <c r="I175" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J175" s="2" t="inlineStr"/>
     </row>
@@ -6685,7 +6685,7 @@
         <v>16.05</v>
       </c>
       <c r="I176" s="2" t="n">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="J176" s="2" t="inlineStr"/>
     </row>
@@ -6717,7 +6717,7 @@
         <v>32.11</v>
       </c>
       <c r="I177" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J177" s="2" t="inlineStr"/>
     </row>
@@ -6753,7 +6753,7 @@
         <v>8.710000000000001</v>
       </c>
       <c r="I178" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J178" s="2" t="inlineStr"/>
     </row>
@@ -6789,7 +6789,7 @@
         <v>10.17</v>
       </c>
       <c r="I179" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J179" s="2" t="inlineStr"/>
     </row>
@@ -6821,7 +6821,7 @@
         <v>16.05</v>
       </c>
       <c r="I180" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J180" s="2" t="inlineStr"/>
     </row>
@@ -6857,7 +6857,7 @@
         <v>7.82</v>
       </c>
       <c r="I181" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J181" s="2" t="inlineStr"/>
     </row>
@@ -6893,7 +6893,7 @@
         <v>8.029999999999999</v>
       </c>
       <c r="I182" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J182" s="2" t="inlineStr"/>
     </row>
@@ -6929,7 +6929,7 @@
         <v>5.26</v>
       </c>
       <c r="I183" s="2" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J183" s="2" t="inlineStr"/>
     </row>
@@ -6965,7 +6965,7 @@
         <v>19.06</v>
       </c>
       <c r="I184" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J184" s="2" t="inlineStr"/>
     </row>
@@ -7001,7 +7001,7 @@
         <v>26.52</v>
       </c>
       <c r="I185" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J185" s="2" t="inlineStr"/>
     </row>
@@ -7033,7 +7033,7 @@
         <v>13.86</v>
       </c>
       <c r="I186" s="2" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J186" s="2" t="inlineStr"/>
     </row>
@@ -7069,7 +7069,7 @@
         <v>3.63</v>
       </c>
       <c r="I187" s="2" t="n">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J187" s="2" t="inlineStr"/>
     </row>
@@ -7105,7 +7105,7 @@
         <v>7.37</v>
       </c>
       <c r="I188" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J188" s="2" t="inlineStr"/>
     </row>
@@ -7141,7 +7141,7 @@
         <v>7.92</v>
       </c>
       <c r="I189" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J189" s="2" t="inlineStr"/>
     </row>
@@ -7177,7 +7177,7 @@
         <v>13.36</v>
       </c>
       <c r="I190" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J190" s="2" t="inlineStr"/>
     </row>
@@ -7213,7 +7213,7 @@
         <v>10.43</v>
       </c>
       <c r="I191" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J191" s="2" t="inlineStr"/>
     </row>
@@ -7249,7 +7249,7 @@
         <v>10.57</v>
       </c>
       <c r="I192" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J192" s="2" t="inlineStr"/>
     </row>
@@ -7285,7 +7285,7 @@
         <v>5.35</v>
       </c>
       <c r="I193" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J193" s="2" t="inlineStr"/>
     </row>
@@ -7321,7 +7321,7 @@
         <v>5.38</v>
       </c>
       <c r="I194" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J194" s="2" t="inlineStr"/>
     </row>
@@ -7357,7 +7357,7 @@
         <v>4.63</v>
       </c>
       <c r="I195" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J195" s="2" t="inlineStr"/>
     </row>
@@ -7393,7 +7393,7 @@
         <v>2.85</v>
       </c>
       <c r="I196" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J196" s="2" t="inlineStr"/>
     </row>
@@ -7429,7 +7429,7 @@
         <v>2.78</v>
       </c>
       <c r="I197" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J197" s="2" t="inlineStr"/>
     </row>
@@ -7465,7 +7465,7 @@
         <v>4.52</v>
       </c>
       <c r="I198" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J198" s="2" t="inlineStr"/>
     </row>
@@ -7501,7 +7501,7 @@
         <v>5.19</v>
       </c>
       <c r="I199" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J199" s="2" t="inlineStr"/>
     </row>
@@ -7533,7 +7533,7 @@
         <v>4.92</v>
       </c>
       <c r="I200" s="2" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J200" s="2" t="inlineStr"/>
     </row>
@@ -7569,7 +7569,7 @@
         <v>6.49</v>
       </c>
       <c r="I201" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J201" s="2" t="inlineStr"/>
     </row>
@@ -7605,7 +7605,7 @@
         <v>6.91</v>
       </c>
       <c r="I202" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J202" s="2" t="inlineStr"/>
     </row>
@@ -7641,7 +7641,7 @@
         <v>7.23</v>
       </c>
       <c r="I203" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J203" s="2" t="inlineStr"/>
     </row>
@@ -7677,7 +7677,7 @@
         <v>14.98</v>
       </c>
       <c r="I204" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J204" s="2" t="inlineStr"/>
     </row>
@@ -7713,7 +7713,7 @@
         <v>37.75</v>
       </c>
       <c r="I205" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J205" s="2" t="inlineStr"/>
     </row>
@@ -7749,7 +7749,7 @@
         <v>20.97</v>
       </c>
       <c r="I206" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J206" s="2" t="inlineStr"/>
     </row>
@@ -7785,7 +7785,7 @@
         <v>12.38</v>
       </c>
       <c r="I207" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J207" s="2" t="inlineStr"/>
     </row>
@@ -7821,7 +7821,7 @@
         <v>10.21</v>
       </c>
       <c r="I208" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J208" s="2" t="inlineStr"/>
     </row>
@@ -7857,7 +7857,7 @@
         <v>11.85</v>
       </c>
       <c r="I209" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J209" s="2" t="inlineStr"/>
     </row>
@@ -7893,7 +7893,7 @@
         <v>14.13</v>
       </c>
       <c r="I210" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J210" s="2" t="inlineStr"/>
     </row>
@@ -7929,7 +7929,7 @@
         <v>17.98</v>
       </c>
       <c r="I211" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J211" s="2" t="inlineStr"/>
     </row>
@@ -7961,7 +7961,7 @@
         <v>6.65</v>
       </c>
       <c r="I212" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J212" s="2" t="inlineStr"/>
     </row>
@@ -7993,7 +7993,7 @@
         <v>5.57</v>
       </c>
       <c r="I213" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J213" s="2" t="inlineStr"/>
     </row>
@@ -8029,7 +8029,7 @@
         <v>6.32</v>
       </c>
       <c r="I214" s="2" t="n">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J214" s="2" t="inlineStr"/>
     </row>
@@ -8065,7 +8065,7 @@
         <v>5.4</v>
       </c>
       <c r="I215" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J215" s="2" t="inlineStr"/>
     </row>
@@ -8101,7 +8101,7 @@
         <v>10.86</v>
       </c>
       <c r="I216" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J216" s="2" t="inlineStr"/>
     </row>
@@ -8137,7 +8137,7 @@
         <v>41.94</v>
       </c>
       <c r="I217" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J217" s="2" t="inlineStr"/>
     </row>
@@ -8173,7 +8173,7 @@
         <v>3.14</v>
       </c>
       <c r="I218" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J218" s="2" t="inlineStr"/>
     </row>
@@ -8209,7 +8209,7 @@
         <v>4.35</v>
       </c>
       <c r="I219" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J219" s="2" t="inlineStr"/>
     </row>
@@ -8241,7 +8241,7 @@
         <v>1705.13</v>
       </c>
       <c r="I220" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J220" s="2" t="inlineStr"/>
     </row>
@@ -8277,7 +8277,7 @@
         <v>12.82</v>
       </c>
       <c r="I221" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J221" s="2" t="inlineStr"/>
     </row>
@@ -8309,7 +8309,7 @@
         <v>56.84</v>
       </c>
       <c r="I222" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J222" s="2" t="inlineStr"/>
     </row>
@@ -8345,7 +8345,7 @@
         <v>31.58</v>
       </c>
       <c r="I223" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J223" s="2" t="inlineStr"/>
     </row>
@@ -8381,7 +8381,7 @@
         <v>32.79</v>
       </c>
       <c r="I224" s="2" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J224" s="2" t="inlineStr"/>
     </row>
@@ -8417,7 +8417,7 @@
         <v>54.13</v>
       </c>
       <c r="I225" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J225" s="2" t="inlineStr"/>
     </row>
@@ -8453,7 +8453,7 @@
         <v>28.9</v>
       </c>
       <c r="I226" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J226" s="2" t="inlineStr"/>
     </row>
@@ -8489,7 +8489,7 @@
         <v>21.86</v>
       </c>
       <c r="I227" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J227" s="2" t="inlineStr"/>
     </row>
@@ -8525,7 +8525,7 @@
         <v>6.45</v>
       </c>
       <c r="I228" s="2" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J228" s="2" t="inlineStr"/>
     </row>
@@ -8561,7 +8561,7 @@
         <v>341</v>
       </c>
       <c r="I229" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J229" s="2" t="inlineStr"/>
     </row>
@@ -8593,7 +8593,7 @@
         <v>568.33</v>
       </c>
       <c r="I230" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J230" s="2" t="inlineStr"/>
     </row>
@@ -8625,7 +8625,7 @@
         <v>1705</v>
       </c>
       <c r="I231" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J231" s="2" t="inlineStr"/>
     </row>
@@ -8661,7 +8661,7 @@
         <v>13.41</v>
       </c>
       <c r="I232" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J232" s="2" t="inlineStr"/>
     </row>
@@ -8697,7 +8697,7 @@
         <v>6.25</v>
       </c>
       <c r="I233" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J233" s="2" t="inlineStr"/>
     </row>
@@ -8733,7 +8733,7 @@
         <v>5.33</v>
       </c>
       <c r="I234" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J234" s="2" t="inlineStr"/>
     </row>
@@ -8769,7 +8769,7 @@
         <v>5.96</v>
       </c>
       <c r="I235" s="2" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J235" s="2" t="inlineStr"/>
     </row>
@@ -8805,7 +8805,7 @@
         <v>13.92</v>
       </c>
       <c r="I236" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J236" s="2" t="inlineStr"/>
     </row>
@@ -8841,7 +8841,7 @@
         <v>3.74</v>
       </c>
       <c r="I237" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J237" s="2" t="inlineStr"/>
     </row>
@@ -8877,7 +8877,7 @@
         <v>5.06</v>
       </c>
       <c r="I238" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J238" s="2" t="inlineStr"/>
     </row>
@@ -8909,7 +8909,7 @@
         <v>735</v>
       </c>
       <c r="I239" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J239" s="2" t="inlineStr"/>
     </row>
@@ -8945,7 +8945,7 @@
         <v>16.28</v>
       </c>
       <c r="I240" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J240" s="2" t="inlineStr"/>
     </row>
@@ -8977,7 +8977,7 @@
         <v>8.01</v>
       </c>
       <c r="I241" s="2" t="n">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="J241" s="2" t="inlineStr"/>
     </row>
@@ -9009,7 +9009,7 @@
         <v>13.56</v>
       </c>
       <c r="I242" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J242" s="2" t="inlineStr"/>
     </row>
@@ -9045,7 +9045,7 @@
         <v>14.65</v>
       </c>
       <c r="I243" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J243" s="2" t="inlineStr"/>
     </row>
@@ -9081,7 +9081,7 @@
         <v>25.26</v>
       </c>
       <c r="I244" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J244" s="2" t="inlineStr"/>
     </row>
@@ -9117,7 +9117,7 @@
         <v>33.3</v>
       </c>
       <c r="I245" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J245" s="2" t="inlineStr"/>
     </row>
@@ -9149,7 +9149,7 @@
         <v>5.47</v>
       </c>
       <c r="I246" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J246" s="2" t="inlineStr"/>
     </row>
@@ -9181,7 +9181,7 @@
         <v>6.91</v>
       </c>
       <c r="I247" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J247" s="2" t="inlineStr"/>
     </row>
@@ -9217,7 +9217,7 @@
         <v>5.69</v>
       </c>
       <c r="I248" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J248" s="2" t="inlineStr"/>
     </row>
@@ -9249,7 +9249,7 @@
         <v>3.94</v>
       </c>
       <c r="I249" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J249" s="2" t="inlineStr"/>
     </row>
@@ -9281,7 +9281,7 @@
         <v>2.74</v>
       </c>
       <c r="I250" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J250" s="2" t="inlineStr"/>
     </row>
@@ -9317,7 +9317,7 @@
         <v>2.56</v>
       </c>
       <c r="I251" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J251" s="2" t="inlineStr"/>
     </row>
@@ -9353,7 +9353,7 @@
         <v>2.8</v>
       </c>
       <c r="I252" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J252" s="2" t="inlineStr"/>
     </row>
@@ -9389,7 +9389,7 @@
         <v>6.74</v>
       </c>
       <c r="I253" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J253" s="2" t="inlineStr"/>
     </row>
@@ -9425,7 +9425,7 @@
         <v>3.7</v>
       </c>
       <c r="I254" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J254" s="2" t="inlineStr"/>
     </row>
@@ -9461,7 +9461,7 @@
         <v>11.49</v>
       </c>
       <c r="I255" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J255" s="2" t="inlineStr"/>
     </row>
@@ -9497,7 +9497,7 @@
         <v>7.46</v>
       </c>
       <c r="I256" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J256" s="2" t="inlineStr"/>
     </row>
@@ -9533,7 +9533,7 @@
         <v>28.08</v>
       </c>
       <c r="I257" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J257" s="2" t="inlineStr"/>
     </row>
@@ -9569,7 +9569,7 @@
         <v>13.07</v>
       </c>
       <c r="I258" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J258" s="2" t="inlineStr"/>
     </row>
@@ -9605,7 +9605,7 @@
         <v>11.66</v>
       </c>
       <c r="I259" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J259" s="2" t="inlineStr"/>
     </row>
@@ -9641,7 +9641,7 @@
         <v>6.61</v>
       </c>
       <c r="I260" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J260" s="2" t="inlineStr"/>
     </row>
@@ -9677,7 +9677,7 @@
         <v>3.09</v>
       </c>
       <c r="I261" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J261" s="2" t="inlineStr"/>
     </row>
@@ -9713,7 +9713,7 @@
         <v>3.35</v>
       </c>
       <c r="I262" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J262" s="2" t="inlineStr"/>
     </row>
@@ -9749,7 +9749,7 @@
         <v>35.84</v>
       </c>
       <c r="I263" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J263" s="2" t="inlineStr"/>
     </row>
@@ -9785,7 +9785,7 @@
         <v>13.59</v>
       </c>
       <c r="I264" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J264" s="2" t="inlineStr"/>
     </row>
@@ -9817,7 +9817,7 @@
         <v>523.84</v>
       </c>
       <c r="I265" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J265" s="2" t="inlineStr"/>
     </row>
@@ -9853,7 +9853,7 @@
         <v>16.06</v>
       </c>
       <c r="I266" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J266" s="2" t="inlineStr"/>
     </row>
@@ -9885,7 +9885,7 @@
         <v>12.46</v>
       </c>
       <c r="I267" s="2" t="n">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J267" s="2" t="inlineStr"/>
     </row>
@@ -9921,7 +9921,7 @@
         <v>23.36</v>
       </c>
       <c r="I268" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J268" s="2" t="inlineStr"/>
     </row>
@@ -9957,7 +9957,7 @@
         <v>4.3</v>
       </c>
       <c r="I269" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J269" s="2" t="inlineStr"/>
     </row>
@@ -9993,7 +9993,7 @@
         <v>5.84</v>
       </c>
       <c r="I270" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J270" s="2" t="inlineStr"/>
     </row>
@@ -10029,7 +10029,7 @@
         <v>1.84</v>
       </c>
       <c r="I271" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J271" s="2" t="inlineStr"/>
     </row>
@@ -10065,7 +10065,7 @@
         <v>1.97</v>
       </c>
       <c r="I272" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J272" s="2" t="inlineStr"/>
     </row>
@@ -10101,7 +10101,7 @@
         <v>8.81</v>
       </c>
       <c r="I273" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J273" s="2" t="inlineStr"/>
     </row>
@@ -10137,7 +10137,7 @@
         <v>7.52</v>
       </c>
       <c r="I274" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J274" s="2" t="inlineStr"/>
     </row>
@@ -10173,7 +10173,7 @@
         <v>6.41</v>
       </c>
       <c r="I275" s="2" t="n">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J275" s="2" t="inlineStr"/>
     </row>
@@ -10209,7 +10209,7 @@
         <v>24.58</v>
       </c>
       <c r="I276" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J276" s="2" t="inlineStr"/>
     </row>
@@ -10245,7 +10245,7 @@
         <v>16.86</v>
       </c>
       <c r="I277" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J277" s="2" t="inlineStr"/>
     </row>
@@ -10281,7 +10281,7 @@
         <v>4.99</v>
       </c>
       <c r="I278" s="2" t="n">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="J278" s="2" t="inlineStr"/>
     </row>
@@ -10317,7 +10317,7 @@
         <v>2.83</v>
       </c>
       <c r="I279" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J279" s="2" t="inlineStr"/>
     </row>
@@ -10353,7 +10353,7 @@
         <v>3.16</v>
       </c>
       <c r="I280" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J280" s="2" t="inlineStr"/>
     </row>
@@ -10385,7 +10385,7 @@
         <v>32.51</v>
       </c>
       <c r="I281" s="2" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J281" s="2" t="inlineStr"/>
     </row>
@@ -10421,7 +10421,7 @@
         <v>17.67</v>
       </c>
       <c r="I282" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J282" s="2" t="inlineStr"/>
     </row>
@@ -10457,7 +10457,7 @@
         <v>23.9</v>
       </c>
       <c r="I283" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J283" s="2" t="inlineStr"/>
     </row>
@@ -10493,7 +10493,7 @@
         <v>5</v>
       </c>
       <c r="I284" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J284" s="2" t="inlineStr"/>
     </row>
@@ -10529,7 +10529,7 @@
         <v>7.02</v>
       </c>
       <c r="I285" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J285" s="2" t="inlineStr"/>
     </row>
@@ -10565,7 +10565,7 @@
         <v>6.79</v>
       </c>
       <c r="I286" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J286" s="2" t="inlineStr"/>
     </row>
@@ -10601,7 +10601,7 @@
         <v>12.02</v>
       </c>
       <c r="I287" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J287" s="2" t="inlineStr"/>
     </row>
@@ -10637,7 +10637,7 @@
         <v>9.57</v>
       </c>
       <c r="I288" s="2" t="n">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="J288" s="2" t="inlineStr"/>
     </row>
@@ -10673,7 +10673,7 @@
         <v>13.74</v>
       </c>
       <c r="I289" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J289" s="2" t="inlineStr"/>
     </row>
@@ -10705,7 +10705,7 @@
         <v>6.7</v>
       </c>
       <c r="I290" s="2" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J290" s="2" t="inlineStr"/>
     </row>
@@ -10741,7 +10741,7 @@
         <v>11.28</v>
       </c>
       <c r="I291" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J291" s="2" t="inlineStr"/>
     </row>
@@ -10777,7 +10777,7 @@
         <v>24.72</v>
       </c>
       <c r="I292" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J292" s="2" t="inlineStr"/>
     </row>
@@ -10813,7 +10813,7 @@
         <v>16.07</v>
       </c>
       <c r="I293" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J293" s="2" t="inlineStr"/>
     </row>
@@ -10849,7 +10849,7 @@
         <v>8.27</v>
       </c>
       <c r="I294" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J294" s="2" t="inlineStr"/>
     </row>
@@ -10885,7 +10885,7 @@
         <v>11.24</v>
       </c>
       <c r="I295" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J295" s="2" t="inlineStr"/>
     </row>
@@ -10921,7 +10921,7 @@
         <v>17.36</v>
       </c>
       <c r="I296" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J296" s="2" t="inlineStr"/>
     </row>
@@ -10957,7 +10957,7 @@
         <v>6.59</v>
       </c>
       <c r="I297" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J297" s="2" t="inlineStr"/>
     </row>
@@ -10989,7 +10989,7 @@
         <v>5.44</v>
       </c>
       <c r="I298" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J298" s="2" t="inlineStr"/>
     </row>
@@ -11025,7 +11025,7 @@
         <v>3.79</v>
       </c>
       <c r="I299" s="2" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J299" s="2" t="inlineStr"/>
     </row>
@@ -11061,7 +11061,7 @@
         <v>8.42</v>
       </c>
       <c r="I300" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J300" s="2" t="inlineStr"/>
     </row>
@@ -11097,7 +11097,7 @@
         <v>27.74</v>
       </c>
       <c r="I301" s="2" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="J301" s="2" t="inlineStr"/>
     </row>
@@ -11133,7 +11133,7 @@
         <v>30.75</v>
       </c>
       <c r="I302" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J302" s="2" t="inlineStr"/>
     </row>
@@ -11169,7 +11169,7 @@
         <v>11.99</v>
       </c>
       <c r="I303" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J303" s="2" t="inlineStr"/>
     </row>
@@ -11205,7 +11205,7 @@
         <v>56.59</v>
       </c>
       <c r="I304" s="2" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J304" s="2" t="inlineStr"/>
     </row>
@@ -11241,7 +11241,7 @@
         <v>14.15</v>
       </c>
       <c r="I305" s="2" t="n">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="J305" s="2" t="inlineStr"/>
     </row>
@@ -11277,7 +11277,7 @@
         <v>34.5</v>
       </c>
       <c r="I306" s="2" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J306" s="2" t="inlineStr"/>
     </row>
@@ -11313,7 +11313,7 @@
         <v>18.61</v>
       </c>
       <c r="I307" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J307" s="2" t="inlineStr"/>
     </row>
@@ -11349,7 +11349,7 @@
         <v>5.66</v>
       </c>
       <c r="I308" s="2" t="n">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J308" s="2" t="inlineStr"/>
     </row>
@@ -11385,7 +11385,7 @@
         <v>15.72</v>
       </c>
       <c r="I309" s="2" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J309" s="2" t="inlineStr"/>
     </row>
@@ -11421,7 +11421,7 @@
         <v>7.72</v>
       </c>
       <c r="I310" s="2" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="J310" s="2" t="inlineStr"/>
     </row>
@@ -11457,7 +11457,7 @@
         <v>19.86</v>
       </c>
       <c r="I311" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J311" s="2" t="inlineStr"/>
     </row>
@@ -11493,7 +11493,7 @@
         <v>13.56</v>
       </c>
       <c r="I312" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J312" s="2" t="inlineStr"/>
     </row>
@@ -11529,7 +11529,7 @@
         <v>10.3</v>
       </c>
       <c r="I313" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J313" s="2" t="inlineStr"/>
     </row>
@@ -11565,7 +11565,7 @@
         <v>17.16</v>
       </c>
       <c r="I314" s="2" t="n">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J314" s="2" t="inlineStr"/>
     </row>
@@ -11601,7 +11601,7 @@
         <v>6.47</v>
       </c>
       <c r="I315" s="2" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J315" s="2" t="inlineStr"/>
     </row>
@@ -11637,7 +11637,7 @@
         <v>5.52</v>
       </c>
       <c r="I316" s="2" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J316" s="2" t="inlineStr"/>
     </row>
@@ -11673,7 +11673,7 @@
         <v>5.25</v>
       </c>
       <c r="I317" s="2" t="n">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="J317" s="2" t="inlineStr"/>
     </row>
@@ -11709,7 +11709,7 @@
         <v>11.44</v>
       </c>
       <c r="I318" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J318" s="2" t="inlineStr"/>
     </row>
@@ -11745,7 +11745,7 @@
         <v>10.53</v>
       </c>
       <c r="I319" s="2" t="n">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="J319" s="2" t="inlineStr"/>
     </row>
@@ -11781,7 +11781,7 @@
         <v>16.95</v>
       </c>
       <c r="I320" s="2" t="n">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="J320" s="2" t="inlineStr"/>
     </row>
@@ -11813,7 +11813,7 @@
         <v>3.28</v>
       </c>
       <c r="I321" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J321" s="2" t="inlineStr"/>
     </row>
@@ -11849,7 +11849,7 @@
         <v>4.06</v>
       </c>
       <c r="I322" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J322" s="2" t="inlineStr"/>
     </row>
@@ -11881,7 +11881,7 @@
         <v>42.23</v>
       </c>
       <c r="I323" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="J323" s="2" t="inlineStr"/>
     </row>
@@ -11913,7 +11913,7 @@
         <v>24.13</v>
       </c>
       <c r="I324" s="2" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="J324" s="2" t="inlineStr"/>
     </row>
@@ -11949,7 +11949,7 @@
         <v>7.57</v>
       </c>
       <c r="I325" s="2" t="n">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J325" s="2" t="inlineStr"/>
     </row>
@@ -11985,7 +11985,7 @@
         <v>11.5</v>
       </c>
       <c r="I326" s="2" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J326" s="2" t="inlineStr"/>
     </row>
@@ -12017,7 +12017,7 @@
         <v>14.61</v>
       </c>
       <c r="I327" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="J327" s="2" t="inlineStr"/>
     </row>
@@ -12053,7 +12053,7 @@
         <v>3.47</v>
       </c>
       <c r="I328" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J328" s="2" t="inlineStr"/>
     </row>
@@ -12089,7 +12089,7 @@
         <v>5.32</v>
       </c>
       <c r="I329" s="2" t="n">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="J329" s="2" t="inlineStr"/>
     </row>

</xml_diff>